<commit_message>
cambios en casa 27 ago2026
</commit_message>
<xml_diff>
--- a/output/semanal/01_perfil_semanal.xlsx
+++ b/output/semanal/01_perfil_semanal.xlsx
@@ -1561,7 +1561,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>exog_nacimientos_indice_semanal</t>
+          <t>exog_semana_anio_sin</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1576,13 +1576,13 @@
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>exog_semana_anio_sin</t>
+          <t>exog_semana_anio_cos</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1597,13 +1597,13 @@
         <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>exog_semana_anio_cos</t>
+          <t>exog_mes_sin</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1618,13 +1618,13 @@
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>exog_mes_sin</t>
+          <t>exog_mes_cos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1645,7 +1645,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>exog_mes_cos</t>
+          <t>exog_nacimientos_indice_publicado_lag_1s</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1660,13 +1660,13 @@
         <v>0</v>
       </c>
       <c r="E55" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>exog_inpc_publicado</t>
+          <t>exog_inpc_publicado_lag_1s</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1687,7 +1687,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>exog_temperatura_lag_1s</t>
+          <t>exog_temperatura_publicado_lag_1s</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">

</xml_diff>